<commit_message>
Lynae -> LynaePeppermint: skirt chains ride the skin's hips, not her leg bones; code-1 leg ratio corrected
The waistline slanted whenever she shifted her weight: each skirt chain was mapped to the skin's
nearest bone (105/107/108/145/102/144), which on the skin's own model carry 0-24% of that spot
while her hips (100/101) carry 40-73%. Every link now takes the bone that drives the same spot of
the skin's own model (nearest vertices, weight-tallied); both rows (3.6 via the renumbering) and
the draft. The card stays on 104.

The code-1 leg ratio of lynaeSheerBake carries the measured remaining gap (0.788/0.872/0.949).
Probes showed no code or mask channel on the skin reaches the legs at all.

Corpus: only the 14 Lynae -> LynaePeppermint outputs changed; blend remaps round-trip; prototype
byte-identical on Lynae11 (117 files); unit tests pass.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/RemapDrafts/LynaeRemapDraft.xlsx
+++ b/Data/RemapDrafts/LynaeRemapDraft.xlsx
@@ -3913,14 +3913,14 @@
         <v>210</v>
       </c>
       <c r="B212" t="n">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="C212" t="n">
         <v>0.4</v>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>REVIEWED: necktie, centre chain: chest (111); the finder put this link on the hips (101) [finder: 101; 132 verts (Component 3) -&gt; 6396 verts (Component 3/Component 4/Component 6), dist 11.1800; runner-up 107 at dist 11.9270]</t>
+          <t>CHANGED 2026-10-12 (111 -&gt; 101): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED: necktie, centre chain: chest (111); the finder put this link on the hips (101) [finder: 101; 132 verts (Component 3) -&gt; 6396 verts (Component 3/Component 4/Component 6), dist 11.1800; runner-up 107 at dist 11.9270]</t>
         </is>
       </c>
     </row>
@@ -3929,14 +3929,14 @@
         <v>211</v>
       </c>
       <c r="B213" t="n">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="C213" t="n">
         <v>0.4</v>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>REVIEWED: necktie, centre chain: chest (111); the finder put this link on the spine (104) [finder: 104; 202 verts (Component 3) -&gt; 3455 verts (Component 3/Component 6), dist 10.4458; runner-up 101 at dist 13.2004]</t>
+          <t>CHANGED 2026-10-12 (111 -&gt; 104): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED: necktie, centre chain: chest (111); the finder put this link on the spine (104) [finder: 104; 202 verts (Component 3) -&gt; 3455 verts (Component 3/Component 6), dist 10.4458; runner-up 101 at dist 13.2004]</t>
         </is>
       </c>
     </row>
@@ -3945,14 +3945,14 @@
         <v>212</v>
       </c>
       <c r="B214" t="n">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="C214" t="n">
         <v>0.4</v>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>REVIEWED: necktie, centre chain: chest (111); the finder put this link on her left breast (126) [finder: 126; 298 verts (Component 3/Component 5) -&gt; 2102 verts (Component 3/Component 6), dist 8.7916; runner-up 122 at dist 9.0537]</t>
+          <t>CHANGED 2026-10-12 (111 -&gt; 104): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED: necktie, centre chain: chest (111); the finder put this link on her left breast (126) [finder: 126; 298 verts (Component 3/Component 5) -&gt; 2102 verts (Component 3/Component 6), dist 8.7916; runner-up 122 at dist 9.0537]</t>
         </is>
       </c>
     </row>
@@ -4217,14 +4217,14 @@
         <v>229</v>
       </c>
       <c r="B231" t="n">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C231" t="n">
         <v>0.304</v>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [322 verts (Component 4) -&gt; 1760 verts (Component 3/Component 4), dist 7.7215; runner-up 101 at dist 11.2395]</t>
+          <t>CHANGED 2026-10-12 (105 -&gt; 101): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [322 verts (Component 4) -&gt; 1760 verts (Component 3/Component 4), dist 7.7215; runner-up 101 at dist 11.2395]</t>
         </is>
       </c>
     </row>
@@ -4233,14 +4233,14 @@
         <v>230</v>
       </c>
       <c r="B232" t="n">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C232" t="n">
         <v>0.755</v>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [214 verts (Component 4) -&gt; 1760 verts (Component 3/Component 4), dist 9.5763; runner-up 107 at dist 12.6191]</t>
+          <t>CHANGED 2026-10-12 (105 -&gt; 101): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [214 verts (Component 4) -&gt; 1760 verts (Component 3/Component 4), dist 9.5763; runner-up 107 at dist 12.6191]</t>
         </is>
       </c>
     </row>
@@ -4249,14 +4249,14 @@
         <v>231</v>
       </c>
       <c r="B233" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="C233" t="n">
         <v>0.217</v>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [452 verts (Component 4) -&gt; 1760 verts (Component 3/Component 4), dist 5.9916; runner-up 108 at dist 12.6235]</t>
+          <t>CHANGED 2026-10-12 (105 -&gt; 100): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [452 verts (Component 4) -&gt; 1760 verts (Component 3/Component 4), dist 5.9916; runner-up 108 at dist 12.6235]</t>
         </is>
       </c>
     </row>
@@ -4377,14 +4377,14 @@
         <v>239</v>
       </c>
       <c r="B241" t="n">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C241" t="n">
         <v>0.5620000000000001</v>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [375 verts (Component 4) -&gt; 1760 verts (Component 3/Component 4), dist 9.5643; runner-up 104 at dist 14.2168]</t>
+          <t>CHANGED 2026-10-12 (105 -&gt; 101): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [375 verts (Component 4) -&gt; 1760 verts (Component 3/Component 4), dist 9.5643; runner-up 104 at dist 14.2168]</t>
         </is>
       </c>
     </row>
@@ -4393,14 +4393,14 @@
         <v>240</v>
       </c>
       <c r="B242" t="n">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C242" t="n">
         <v>0.467</v>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [603 verts (Component 4) -&gt; 1760 verts (Component 3/Component 4), dist 6.9485; runner-up 107 at dist 14.2503]</t>
+          <t>CHANGED 2026-10-12 (105 -&gt; 101): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [603 verts (Component 4) -&gt; 1760 verts (Component 3/Component 4), dist 6.9485; runner-up 107 at dist 14.2503]</t>
         </is>
       </c>
     </row>
@@ -4409,14 +4409,14 @@
         <v>241</v>
       </c>
       <c r="B243" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="C243" t="n">
         <v>0.3</v>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>REVIEWED: pleated skirt, left side (LynaePeppermint wears shorts): her left side-hip helper (108), like 246 / 248 / 255; the finder's 104 is the spine, 13 units away [finder: 104; 475 verts (Component 4) -&gt; 3455 verts (Component 3/Component 6), dist 14.3631; runner-up 108 at dist 11.5247; in chain 241-242 -&gt; 104-105]</t>
+          <t>CHANGED 2026-10-12 (108 -&gt; 100): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED: pleated skirt, left side (LynaePeppermint wears shorts): her left side-hip helper (108), like 246 / 248 / 255; the finder's 104 is the spine, 13 units away [finder: 104; 475 verts (Component 4) -&gt; 3455 verts (Component 3/Component 6), dist 14.3631; runner-up 108 at dist 11.5247; in chain 241-242 -&gt; 104-105]</t>
         </is>
       </c>
     </row>
@@ -4425,14 +4425,14 @@
         <v>242</v>
       </c>
       <c r="B244" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="C244" t="n">
         <v>0.035</v>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [723 verts (Component 4) -&gt; 1760 verts (Component 3/Component 4), dist 2.3646; runner-up 108 at dist 9.9053; in chain 241-242 -&gt; 104-105]</t>
+          <t>CHANGED 2026-10-12 (105 -&gt; 100): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [723 verts (Component 4) -&gt; 1760 verts (Component 3/Component 4), dist 2.3646; runner-up 108 at dist 9.9053; in chain 241-242 -&gt; 104-105]</t>
         </is>
       </c>
     </row>
@@ -4441,14 +4441,14 @@
         <v>243</v>
       </c>
       <c r="B245" t="n">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="C245" t="n">
         <v>0.148</v>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [440 verts (Component 4) -&gt; 3502 verts (Component 3/Component 4), dist 4.2767; runner-up 101 at dist 7.7068]</t>
+          <t>CHANGED 2026-10-12 (107 -&gt; 100): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [440 verts (Component 4) -&gt; 3502 verts (Component 3/Component 4), dist 4.2767; runner-up 101 at dist 7.7068]</t>
         </is>
       </c>
     </row>
@@ -4457,14 +4457,14 @@
         <v>244</v>
       </c>
       <c r="B246" t="n">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="C246" t="n">
         <v>0.121</v>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [634 verts (Component 4) -&gt; 3502 verts (Component 3/Component 4), dist 3.6253; runner-up 101 at dist 9.8726]</t>
+          <t>CHANGED 2026-10-12 (107 -&gt; 100): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [634 verts (Component 4) -&gt; 3502 verts (Component 3/Component 4), dist 3.6253; runner-up 101 at dist 9.8726]</t>
         </is>
       </c>
     </row>
@@ -4473,14 +4473,14 @@
         <v>245</v>
       </c>
       <c r="B247" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C247" t="n">
         <v>0.3</v>
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>REVIEWED: pleated skirt, back left: her left buttock helper (102), like 262 / 264 / 308; the finder sent it onto her JACKET's hem chain (221), a different garment's physics [finder: 221; 179 verts (Component 4) -&gt; 853 verts (Component 4/Component 5), dist 8.5984; runner-up 220 at dist 12.0260]</t>
+          <t>CHANGED 2026-10-12 (102 -&gt; 100): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED: pleated skirt, back left: her left buttock helper (102), like 262 / 264 / 308; the finder sent it onto her JACKET's hem chain (221), a different garment's physics [finder: 221; 179 verts (Component 4) -&gt; 853 verts (Component 4/Component 5), dist 8.5984; runner-up 220 at dist 12.0260]</t>
         </is>
       </c>
     </row>
@@ -4489,14 +4489,14 @@
         <v>246</v>
       </c>
       <c r="B248" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="C248" t="n">
         <v>0.8090000000000001</v>
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [326 verts (Component 4) -&gt; 1036 verts (Component 3/Component 4), dist 11.6184; runner-up 115 at dist 12.2452]</t>
+          <t>CHANGED 2026-10-12 (108 -&gt; 100): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [326 verts (Component 4) -&gt; 1036 verts (Component 3/Component 4), dist 11.6184; runner-up 115 at dist 12.2452]</t>
         </is>
       </c>
     </row>
@@ -4521,14 +4521,14 @@
         <v>248</v>
       </c>
       <c r="B250" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="C250" t="n">
         <v>0.5629999999999999</v>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [386 verts (Component 4) -&gt; 1036 verts (Component 3/Component 4), dist 6.0827; runner-up 105 at dist 10.7346]</t>
+          <t>CHANGED 2026-10-12 (108 -&gt; 100): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [386 verts (Component 4) -&gt; 1036 verts (Component 3/Component 4), dist 6.0827; runner-up 105 at dist 10.7346]</t>
         </is>
       </c>
     </row>
@@ -4537,14 +4537,14 @@
         <v>249</v>
       </c>
       <c r="B251" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C251" t="n">
         <v>0.3</v>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>REVIEWED: pleated skirt, back left: her left buttock helper (102); the finder sent it onto her JACKET's hem chain (216) [finder: 216; 381 verts (Component 4) -&gt; 633 verts (Component 4/Component 5), dist 8.2690; runner-up 211 at dist 11.5104]</t>
+          <t>CHANGED 2026-10-12 (102 -&gt; 100): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED: pleated skirt, back left: her left buttock helper (102); the finder sent it onto her JACKET's hem chain (216) [finder: 216; 381 verts (Component 4) -&gt; 633 verts (Component 4/Component 5), dist 8.2690; runner-up 211 at dist 11.5104]</t>
         </is>
       </c>
     </row>
@@ -4553,14 +4553,14 @@
         <v>250</v>
       </c>
       <c r="B252" t="n">
-        <v>144</v>
+        <v>100</v>
       </c>
       <c r="C252" t="n">
         <v>0.3</v>
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>REVIEWED: pleated skirt, back right: her right buttock helper (144), like 260 / 261 / 321; the finder sent it onto her JACKET's hem chain (212) [finder: 212; 347 verts (Component 4) -&gt; 1562 verts (Component 4/Component 5), dist 9.9830; runner-up 214 at dist 10.2600]</t>
+          <t>CHANGED 2026-10-12 (144 -&gt; 100): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED: pleated skirt, back right: her right buttock helper (144), like 260 / 261 / 321; the finder sent it onto her JACKET's hem chain (212) [finder: 212; 347 verts (Component 4) -&gt; 1562 verts (Component 4/Component 5), dist 9.9830; runner-up 214 at dist 10.2600]</t>
         </is>
       </c>
     </row>
@@ -4569,14 +4569,14 @@
         <v>251</v>
       </c>
       <c r="B253" t="n">
-        <v>144</v>
+        <v>100</v>
       </c>
       <c r="C253" t="n">
         <v>0.3</v>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>REVIEWED: pleated skirt, back right: her right buttock helper (144); the finder sent it onto her JACKET's hem chain (214) [finder: 214; 101 verts (Component 4) -&gt; 1524 verts (Component 4/Component 5), dist 10.8928; runner-up 215 at dist 12.8727]</t>
+          <t>CHANGED 2026-10-12 (144 -&gt; 100): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED: pleated skirt, back right: her right buttock helper (144); the finder sent it onto her JACKET's hem chain (214) [finder: 214; 101 verts (Component 4) -&gt; 1524 verts (Component 4/Component 5), dist 10.8928; runner-up 215 at dist 12.8727]</t>
         </is>
       </c>
     </row>
@@ -4585,14 +4585,14 @@
         <v>252</v>
       </c>
       <c r="B254" t="n">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="C254" t="n">
         <v>0.703</v>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [94 verts (Component 4) -&gt; 3502 verts (Component 3/Component 4), dist 7.8763; runner-up 101 at dist 8.9179]</t>
+          <t>CHANGED 2026-10-12 (107 -&gt; 101): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [94 verts (Component 4) -&gt; 3502 verts (Component 3/Component 4), dist 7.8763; runner-up 101 at dist 8.9179]</t>
         </is>
       </c>
     </row>
@@ -4601,14 +4601,14 @@
         <v>253</v>
       </c>
       <c r="B255" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C255" t="n">
         <v>0.894</v>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [744 verts (Component 4) -&gt; 3502 verts (Component 3/Component 4), dist 9.1535; runner-up 106 at dist 9.4832]</t>
+          <t>CHANGED 2026-10-12 (107 -&gt; 106): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [744 verts (Component 4) -&gt; 3502 verts (Component 3/Component 4), dist 9.1535; runner-up 106 at dist 9.4832]</t>
         </is>
       </c>
     </row>
@@ -4617,14 +4617,14 @@
         <v>254</v>
       </c>
       <c r="B256" t="n">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C256" t="n">
         <v>0.5620000000000001</v>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [735 verts (Component 4) -&gt; 1760 verts (Component 3/Component 4), dist 7.1194; runner-up 103 at dist 8.8228]</t>
+          <t>CHANGED 2026-10-12 (105 -&gt; 103): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [735 verts (Component 4) -&gt; 1760 verts (Component 3/Component 4), dist 7.1194; runner-up 103 at dist 8.8228]</t>
         </is>
       </c>
     </row>
@@ -4633,14 +4633,14 @@
         <v>255</v>
       </c>
       <c r="B257" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="C257" t="n">
         <v>0.14</v>
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [523 verts (Component 4) -&gt; 1036 verts (Component 3/Component 4), dist 2.1410; runner-up 105 at dist 9.9737]</t>
+          <t>CHANGED 2026-10-12 (108 -&gt; 100): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [523 verts (Component 4) -&gt; 1036 verts (Component 3/Component 4), dist 2.1410; runner-up 105 at dist 9.9737]</t>
         </is>
       </c>
     </row>
@@ -4649,14 +4649,14 @@
         <v>256</v>
       </c>
       <c r="B258" t="n">
-        <v>145</v>
+        <v>100</v>
       </c>
       <c r="C258" t="n">
         <v>0.79</v>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [131 verts (Component 4) -&gt; 1047 verts (Component 3/Component 4), dist 10.1193; runner-up 107 at dist 10.8157]</t>
+          <t>CHANGED 2026-10-12 (145 -&gt; 100): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [131 verts (Component 4) -&gt; 1047 verts (Component 3/Component 4), dist 10.1193; runner-up 107 at dist 10.8157]</t>
         </is>
       </c>
     </row>
@@ -4665,14 +4665,14 @@
         <v>257</v>
       </c>
       <c r="B259" t="n">
-        <v>145</v>
+        <v>106</v>
       </c>
       <c r="C259" t="n">
         <v>0.533</v>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [659 verts (Component 4) -&gt; 1047 verts (Component 3/Component 4), dist 6.2113; runner-up 144 at dist 11.0251]</t>
+          <t>CHANGED 2026-10-12 (145 -&gt; 106): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [659 verts (Component 4) -&gt; 1047 verts (Component 3/Component 4), dist 6.2113; runner-up 144 at dist 11.0251]</t>
         </is>
       </c>
     </row>
@@ -4681,14 +4681,14 @@
         <v>258</v>
       </c>
       <c r="B260" t="n">
-        <v>145</v>
+        <v>100</v>
       </c>
       <c r="C260" t="n">
         <v>0.109</v>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [522 verts (Component 4) -&gt; 1047 verts (Component 3/Component 4), dist 2.1017; runner-up 144 at dist 11.6031]</t>
+          <t>CHANGED 2026-10-12 (145 -&gt; 100): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [522 verts (Component 4) -&gt; 1047 verts (Component 3/Component 4), dist 2.1017; runner-up 144 at dist 11.6031]</t>
         </is>
       </c>
     </row>
@@ -4697,14 +4697,14 @@
         <v>259</v>
       </c>
       <c r="B261" t="n">
-        <v>145</v>
+        <v>100</v>
       </c>
       <c r="C261" t="n">
         <v>0.261</v>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [337 verts (Component 4) -&gt; 1047 verts (Component 3/Component 4), dist 5.3780; runner-up 107 at dist 9.3436]</t>
+          <t>CHANGED 2026-10-12 (145 -&gt; 100): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [337 verts (Component 4) -&gt; 1047 verts (Component 3/Component 4), dist 5.3780; runner-up 107 at dist 9.3436]</t>
         </is>
       </c>
     </row>
@@ -4713,14 +4713,14 @@
         <v>260</v>
       </c>
       <c r="B262" t="n">
-        <v>144</v>
+        <v>100</v>
       </c>
       <c r="C262" t="n">
         <v>0.294</v>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [490 verts (Component 4) -&gt; 744 verts (Component 3/Component 4), dist 6.4563; runner-up 213 at dist 10.0744]</t>
+          <t>CHANGED 2026-10-12 (144 -&gt; 100): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [490 verts (Component 4) -&gt; 744 verts (Component 3/Component 4), dist 6.4563; runner-up 213 at dist 10.0744]</t>
         </is>
       </c>
     </row>
@@ -4729,14 +4729,14 @@
         <v>261</v>
       </c>
       <c r="B263" t="n">
-        <v>144</v>
+        <v>100</v>
       </c>
       <c r="C263" t="n">
         <v>0.128</v>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [638 verts (Component 4) -&gt; 744 verts (Component 3/Component 4), dist 3.8589; runner-up 213 at dist 9.9405]</t>
+          <t>CHANGED 2026-10-12 (144 -&gt; 100): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [638 verts (Component 4) -&gt; 744 verts (Component 3/Component 4), dist 3.8589; runner-up 213 at dist 9.9405]</t>
         </is>
       </c>
     </row>
@@ -4745,14 +4745,14 @@
         <v>262</v>
       </c>
       <c r="B264" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C264" t="n">
         <v>0.854</v>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [505 verts (Component 4) -&gt; 764 verts (Component 3/Component 4), dist 6.0165; runner-up 216 at dist 6.4452; in chain 262-263 -&gt; 102-103]</t>
+          <t>CHANGED 2026-10-12 (102 -&gt; 100): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [505 verts (Component 4) -&gt; 764 verts (Component 3/Component 4), dist 6.0165; runner-up 216 at dist 6.4452; in chain 262-263 -&gt; 102-103]</t>
         </is>
       </c>
     </row>
@@ -4761,14 +4761,14 @@
         <v>263</v>
       </c>
       <c r="B265" t="n">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="C265" t="n">
         <v>0.3</v>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>REVIEWED: pleated skirt, left side hem: her left side-hip helper (108), the twin of 257 -&gt; 145; the finder's 103 is the thigh, which bends the hem with every step [finder: 103; 650 verts (Component 4) -&gt; 2915 verts (Component 3/Component 4), dist 8.8470; runner-up 108 at dist 5.9301; in chain 262-263 -&gt; 102-103]</t>
+          <t>CHANGED 2026-10-12 (108 -&gt; 103): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED: pleated skirt, left side hem: her left side-hip helper (108), the twin of 257 -&gt; 145; the finder's 103 is the thigh, which bends the hem with every step [finder: 103; 650 verts (Component 4) -&gt; 2915 verts (Component 3/Component 4), dist 8.8470; runner-up 108 at dist 5.9301; in chain 262-263 -&gt; 102-103]</t>
         </is>
       </c>
     </row>
@@ -4777,14 +4777,14 @@
         <v>264</v>
       </c>
       <c r="B266" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C266" t="n">
         <v>0.622</v>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [636 verts (Component 4) -&gt; 764 verts (Component 3/Component 4), dist 4.0915; runner-up 208 at dist 5.4935]</t>
+          <t>CHANGED 2026-10-12 (102 -&gt; 100): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [636 verts (Component 4) -&gt; 764 verts (Component 3/Component 4), dist 4.0915; runner-up 208 at dist 5.4935]</t>
         </is>
       </c>
     </row>
@@ -4825,14 +4825,14 @@
         <v>267</v>
       </c>
       <c r="B269" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C269" t="n">
         <v>0.991</v>
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [426 verts (Component 4) -&gt; 3502 verts (Component 3/Component 4), dist 7.8702; runner-up 106 at dist 7.8957]</t>
+          <t>CHANGED 2026-10-12 (107 -&gt; 106): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [426 verts (Component 4) -&gt; 3502 verts (Component 3/Component 4), dist 7.8702; runner-up 106 at dist 7.8957]</t>
         </is>
       </c>
     </row>
@@ -5369,14 +5369,14 @@
         <v>301</v>
       </c>
       <c r="B303" t="n">
-        <v>145</v>
+        <v>106</v>
       </c>
       <c r="C303" t="n">
         <v>0.242</v>
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [424 verts (Component 4) -&gt; 1047 verts (Component 3/Component 4), dist 3.7743; runner-up 106 at dist 7.9622]</t>
+          <t>CHANGED 2026-10-12 (145 -&gt; 106): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [424 verts (Component 4) -&gt; 1047 verts (Component 3/Component 4), dist 3.7743; runner-up 106 at dist 7.9622]</t>
         </is>
       </c>
     </row>
@@ -5433,14 +5433,14 @@
         <v>305</v>
       </c>
       <c r="B307" t="n">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C307" t="n">
         <v>0.131</v>
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [194 verts (Component 4) -&gt; 1760 verts (Component 3/Component 4), dist 4.4075; runner-up 103 at dist 7.4941; in chain 305-306 -&gt; 105-106]</t>
+          <t>CHANGED 2026-10-12 (105 -&gt; 103): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [194 verts (Component 4) -&gt; 1760 verts (Component 3/Component 4), dist 4.4075; runner-up 103 at dist 7.4941; in chain 305-306 -&gt; 105-106]</t>
         </is>
       </c>
     </row>
@@ -5465,14 +5465,14 @@
         <v>307</v>
       </c>
       <c r="B309" t="n">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="C309" t="n">
         <v>0.192</v>
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [299 verts (Component 4) -&gt; 1036 verts (Component 3/Component 4), dist 3.3456; runner-up 103 at dist 7.5075]</t>
+          <t>CHANGED 2026-10-12 (108 -&gt; 103): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [299 verts (Component 4) -&gt; 1036 verts (Component 3/Component 4), dist 3.3456; runner-up 103 at dist 7.5075]</t>
         </is>
       </c>
     </row>
@@ -5481,14 +5481,14 @@
         <v>308</v>
       </c>
       <c r="B310" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C310" t="n">
         <v>0.094</v>
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [321 verts (Component 4) -&gt; 764 verts (Component 3/Component 4), dist 2.0754; runner-up 208 at dist 9.0567]</t>
+          <t>CHANGED 2026-10-12 (102 -&gt; 100): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [321 verts (Component 4) -&gt; 764 verts (Component 3/Component 4), dist 2.0754; runner-up 208 at dist 9.0567]</t>
         </is>
       </c>
     </row>
@@ -5689,14 +5689,14 @@
         <v>321</v>
       </c>
       <c r="B323" t="n">
-        <v>144</v>
+        <v>100</v>
       </c>
       <c r="C323" t="n">
         <v>0.042</v>
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [401 verts (Component 4) -&gt; 744 verts (Component 3/Component 4), dist 2.3797; runner-up 213 at dist 11.7470]</t>
+          <t>CHANGED 2026-10-12 (144 -&gt; 100): the waistline slanted on LynaePeppermint when she shifted her weight. Her skirt chains rode the skin's leg-driven bones, which carry 0-24% of that spot on the skin's own model; the target is now the bone that drives the same spot of the skin's own model (nearest vertices, weighted). | was: REVIEWED, kept: BEHAVIOUR: pleated skirt panel. LynaePeppermint wears shorts, so the panel rides her hip helper bone on the same side (front / side / back), which the game drives partly from the thigh: the skirt follows the legs the way her shorts do instead of swinging, and never rides her jacket's physics. Watch the front panels when she steps [401 verts (Component 4) -&gt; 744 verts (Component 3/Component 4), dist 2.3797; runner-up 213 at dist 11.7470]</t>
         </is>
       </c>
     </row>

</xml_diff>